<commit_message>
Actualizando direccion comercial en el membrete del presupuesto
</commit_message>
<xml_diff>
--- a/plantilla_presupuesto.xlsx
+++ b/plantilla_presupuesto.xlsx
@@ -35,13 +35,7 @@
     <t>DICAD AMERICA SAS</t>
   </si>
   <si>
-    <t>Agustín Piaggio 822, Mz.: 24</t>
-  </si>
-  <si>
     <t>Córdoba</t>
-  </si>
-  <si>
-    <t>CP: 5014</t>
   </si>
   <si>
     <t>Argentina</t>
@@ -142,6 +136,12 @@
   </si>
   <si>
     <t>*******</t>
+  </si>
+  <si>
+    <t>Lisandro de la Torre N° 747,VCP.</t>
+  </si>
+  <si>
+    <t>CP: 5152</t>
   </si>
 </sst>
 </file>
@@ -576,13 +576,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>11616</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>1231280</xdr:colOff>
+      <xdr:colOff>1219664</xdr:colOff>
       <xdr:row>38</xdr:row>
       <xdr:rowOff>127774</xdr:rowOff>
     </xdr:to>
@@ -607,7 +607,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="11616" y="0"/>
+          <a:off x="0" y="0"/>
           <a:ext cx="9827012" cy="11360304"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -955,48 +955,48 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="24" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="24" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="24" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="24" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="24" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="14" spans="1:6" ht="19.5" thickBot="1" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>0</v>
@@ -1005,13 +1005,13 @@
         <v>1</v>
       </c>
       <c r="D14" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="6" t="s">
         <v>11</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -1020,31 +1020,31 @@
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F15" s="7" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="17" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A17" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B17" s="9" t="s">
+      <c r="F17" s="10" t="s">
         <v>15</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:6" s="12" customFormat="1" ht="110.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1081,25 +1081,25 @@
     </row>
     <row r="22" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="E22" s="23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="F22" s="23"/>
     </row>
     <row r="23" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="E23" s="15" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F23" s="15"/>
     </row>
     <row r="24" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="E24" s="16" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="F24" s="16"/>
     </row>
     <row r="25" spans="1:6" s="14" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E25" s="17" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F25" s="17"/>
     </row>
@@ -1109,7 +1109,7 @@
     <row r="29" spans="1:6" s="14" customFormat="1" x14ac:dyDescent="0.25"/>
     <row r="30" spans="1:6" s="14" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A30" s="26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B30" s="27"/>
       <c r="C30" s="27"/>
@@ -1118,7 +1118,7 @@
     </row>
     <row r="35" spans="1:6" ht="18.75" x14ac:dyDescent="0.4">
       <c r="A35" s="18" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B35" s="19"/>
       <c r="C35" s="20"/>
@@ -1134,7 +1134,7 @@
     </row>
     <row r="38" spans="1:6" ht="15.75" x14ac:dyDescent="0.3">
       <c r="B38" s="22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>